<commit_message>
Fix remaining codebook violations in arrete09311 and decret20101281
Correct policy_target E/F, lifecycle phases L, instrument stages Q, and
budget text N when M=0. CENPOLMAR exclusion file now headers-only (no
invalid partial instrument row). Full inventory validates with 0 issues.

Co-authored-by: Vaibhav <shivrain@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/4P_Index_Arrete_09311_Huiles_Usees.xlsx
+++ b/4P_Index_Arrete_09311_Huiles_Usees.xlsx
@@ -625,11 +625,11 @@
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>use, collection, disposal</t>
+          <t>consumption, disposal, environmental leakage</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
@@ -722,11 +722,11 @@
         </is>
       </c>
       <c r="K3" s="2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>use, collection, disposal</t>
+          <t>consumption, disposal, environmental leakage</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
@@ -746,7 +746,7 @@
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Disposal</t>
+          <t>End of life</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
@@ -819,11 +819,11 @@
         </is>
       </c>
       <c r="K4" s="2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>use, collection, disposal</t>
+          <t>consumption, disposal, environmental leakage</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">

</xml_diff>